<commit_message>
Add manual and troubleshooting
</commit_message>
<xml_diff>
--- a/CS_Checklist.xlsx
+++ b/CS_Checklist.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -846,7 +846,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>통합</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -856,12 +856,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>클라이언트 2번 조명 이물 확인 후 클리닝</t>
+          <t>파단 이후 클리닝</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Check and Clean Client #2 Lighting for Dust/Tiny Particles</t>
+          <t>Cleaning After Break</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>탈리(Delamination)</t>
+          <t>통합</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -886,12 +886,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>탈리비전 즉정지 알람 시 작업자 스크랩 조치 확인</t>
+          <t>클라이언트 2번 조명 이물 확인 후 클리닝</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Verify Operator Scrap Action on Delamination Vision Stop Alarm</t>
+          <t>Check and Clean Client #2 Lighting for Dust/Tiny Particles</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -901,27 +901,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>양극</t>
+          <t>음극</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>탈리(Delamination)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>정합성</t>
+          <t>H/W &amp; 클리닝</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>탭 접어서 통합비전/마킹비전 셀 ID 매칭 확인</t>
+          <t>탈리비전 즉정지 알람 시 작업자 스크랩 조치 확인</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fold tab and check Cell ID matching (Integrated/Marking Vision)</t>
+          <t>Verify Operator Scrap Action on Delamination Vision Stop Alarm</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -946,12 +946,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>엔코더 슬립 체크</t>
+          <t>탭 접어서 통합비전/마킹비전 셀 ID 매칭 확인</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Check Encoder Slip</t>
+          <t>Fold tab and check Cell ID matching (Integrated/Marking Vision)</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -976,12 +976,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>트리거 보드 신호 체크</t>
+          <t>엔코더 슬립 체크</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Check Trigger Board Signal</t>
+          <t>Check Encoder Slip</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1001,17 +1001,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>S/W</t>
+          <t>정합성</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>비전 프로그램 그래프 및 측정 데이터 확인</t>
+          <t>트리거 보드 신호 체크</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Check Vision Program Graphs &amp; Measurement Data</t>
+          <t>Check Trigger Board Signal</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1036,12 +1036,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>검사항목 데이터 이미지 정상 출력 확인</t>
+          <t>비전 프로그램 그래프 및 측정 데이터 확인</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Check Inspection Item Data &amp; Image Output</t>
+          <t>Check Vision Program Graphs &amp; Measurement Data</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CSV 파일 생성 여부 확인</t>
+          <t>검사항목 데이터 이미지 정상 출력 확인</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Verify CSV File Creation</t>
+          <t>Check Inspection Item Data &amp; Image Output</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1096,12 +1096,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SPC+ 통신 연동 체크</t>
+          <t>CSV 파일 생성 여부 확인</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Check SPC+ Communication Link</t>
+          <t>Verify CSV File Creation</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>메모리 점유율 및 PC 상태 체크</t>
+          <t>SPC+ 통신 연동 체크</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Check Memory Usage &amp; PC Status</t>
+          <t>Check SPC+ Communication Link</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PC 시간 동기화 확인</t>
+          <t>메모리 점유율 및 PC 상태 체크</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Verify PC Time Synchronization</t>
+          <t>Check Memory Usage &amp; PC Status</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1181,17 +1181,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>H/W &amp; 클리닝</t>
+          <t>S/W</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>조명 상태 및 점등 확인</t>
+          <t>PC 시간 동기화 확인</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Check Lighting Status &amp; Illumination</t>
+          <t>Verify PC Time Synchronization</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1216,12 +1216,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>카메라 착상 및 고정 상태 확인</t>
+          <t>조명 상태 및 점등 확인</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Check Camera Mounting &amp; Fixation</t>
+          <t>Check Lighting Status &amp; Illumination</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1246,12 +1246,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>탭 센서 및 탭 가이드 이물 확인 및 클리닝</t>
+          <t>카메라 착상 및 고정 상태 확인</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Check/Clean Tab Sensor &amp; Tab Guide (Dust/Tiny Particles)</t>
+          <t>Check Camera Mounting &amp; Fixation</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1276,12 +1276,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>롤러(Roller) 클리닝</t>
+          <t>탭 센서 및 탭 가이드 이물 확인 및 클리닝</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Clean Roller</t>
+          <t>Check/Clean Tab Sensor &amp; Tab Guide (Dust/Tiny Particles)</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1296,25 +1296,85 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>H/W &amp; 클리닝</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>롤러(Roller) 클리닝</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Clean Roller</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>양극</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>H/W &amp; 클리닝</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>파단 이후 클리닝</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Cleaning After Break</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>양극</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>통합</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>H/W &amp; 클리닝</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>클라이언트 2번 조명 이물 확인 후 클리닝</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Check and Clean Client #2 Lighting for Dust/Tiny Particles</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="F32" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>